<commit_message>
Fix file locking, elapsed time, charts, Firestore upload
</commit_message>
<xml_diff>
--- a/ci_output/ci_report.xlsx
+++ b/ci_output/ci_report.xlsx
@@ -110,7 +110,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -118,6 +117,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -233,7 +233,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Overall WER, CER, SER and S / D / I</a:t>
+              <a:t>Accuracy: WER, CER and SER</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -254,12 +254,112 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Summary'!$R$4:$R$9</f>
+              <f>'Summary'!$R$4:$R$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$S$4:$S$9</f>
+              <f>'Summary'!$S$4:$S$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="100"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>percent</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Error counts: substitutions, deletions, insertions</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$R$9:$R$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$S$9:$S$11</f>
             </numRef>
           </val>
         </ser>
@@ -302,7 +402,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>percent  /  words</a:t>
+                  <a:t>words</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -328,7 +428,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="3960000"/>
+    <ext cx="6120000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -338,6 +438,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -644,7 +766,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="3" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -657,19 +779,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>results_detailed_20261016_153135.csv   |   9 samples scored, 1 failed, 10 attempted</t>
+          <t>results_detailed_20261028_175106.csv   |   9 samples scored, 1 failed, 10 attempted</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>Measure</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>Value</t>
+          <t>Accuracy</t>
         </is>
       </c>
     </row>
@@ -729,78 +846,75 @@
           <t>Meaning</t>
         </is>
       </c>
-      <c r="R7" s="4" t="inlineStr">
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Average WER %</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>26.83</v>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Mean of the individual sample WERs.</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>Error counts</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Average CER %</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Character error rate, averaged per sample.</t>
+        </is>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
         <is>
           <t>Substitutions</t>
         </is>
       </c>
-      <c r="S7" s="7" t="n">
+      <c r="S9" s="10" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>Average WER %</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>26.83</v>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Mean of the individual sample WERs.</t>
-        </is>
-      </c>
-      <c r="R8" s="4" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>SER %</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>77.78</v>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Share of samples with at least one error.</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
         <is>
           <t>Deletions</t>
         </is>
       </c>
-      <c r="S8" s="7" t="n">
+      <c r="S10" s="10" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Average CER %</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n">
-        <v>23.4</v>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Character error rate, averaged per sample.</t>
-        </is>
-      </c>
-      <c r="R9" s="4" t="inlineStr">
-        <is>
-          <t>Insertions</t>
-        </is>
-      </c>
-      <c r="S9" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>SER %</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="n">
-        <v>77.78</v>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Share of samples with at least one error.</t>
-        </is>
-      </c>
-    </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Substitutions</t>
         </is>
@@ -808,14 +922,22 @@
       <c r="B11" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Reference word replaced by a different word.</t>
         </is>
       </c>
+      <c r="R11" s="4" t="inlineStr">
+        <is>
+          <t>Insertions</t>
+        </is>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Deletions</t>
         </is>
@@ -823,14 +945,14 @@
       <c r="B12" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Reference word missing from the output.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Insertions</t>
         </is>
@@ -838,14 +960,14 @@
       <c r="B13" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Extra word the recogniser added.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Reference words</t>
         </is>
@@ -853,14 +975,14 @@
       <c r="B14" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Total words scored against.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Samples scored</t>
         </is>
@@ -868,14 +990,14 @@
       <c r="B15" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Excludes failed and empty samples.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Samples failed</t>
         </is>
@@ -883,7 +1005,7 @@
       <c r="B16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Counted, never averaged into accuracy.</t>
         </is>

</xml_diff>